<commit_message>
added fake CEO names and contact numbers
</commit_message>
<xml_diff>
--- a/orgs_test/2023-11-21 fictional_orgs_list.xlsx
+++ b/orgs_test/2023-11-21 fictional_orgs_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin.ingram/Martin Ingram R Work/martin-ingram.github.io/orgs_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B78D3E2-96E2-924C-B572-8E30050599EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD0818C-9DA2-2F47-BED3-3B0438EE9D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31620" yWindow="2080" windowWidth="28040" windowHeight="17180" xr2:uid="{9B7B9A65-6A20-384F-90D3-B47F15698559}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" xr2:uid="{9B7B9A65-6A20-384F-90D3-B47F15698559}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="203">
   <si>
     <t>Stark Industries</t>
   </si>
@@ -372,13 +372,286 @@
   </si>
   <si>
     <t>Sony</t>
+  </si>
+  <si>
+    <t>Ethan Lee</t>
+  </si>
+  <si>
+    <t>Olivia Martin</t>
+  </si>
+  <si>
+    <t>Jayden Smith</t>
+  </si>
+  <si>
+    <t>Isabella Patel</t>
+  </si>
+  <si>
+    <t>Michael Johnson</t>
+  </si>
+  <si>
+    <t>Sophia Davis</t>
+  </si>
+  <si>
+    <t>Liam Brown</t>
+  </si>
+  <si>
+    <t>Emily Wilson</t>
+  </si>
+  <si>
+    <t>Jacob Miller</t>
+  </si>
+  <si>
+    <t>Ava Lopez</t>
+  </si>
+  <si>
+    <t>William Moore</t>
+  </si>
+  <si>
+    <t>Mia Taylor</t>
+  </si>
+  <si>
+    <t>Noah Anderson</t>
+  </si>
+  <si>
+    <t>Lily Thomas</t>
+  </si>
+  <si>
+    <t>James Jackson</t>
+  </si>
+  <si>
+    <t>Amelia Harris</t>
+  </si>
+  <si>
+    <t>Logan Martinez</t>
+  </si>
+  <si>
+    <t>Charlotte Clark</t>
+  </si>
+  <si>
+    <t>Benjamin Rodriguez</t>
+  </si>
+  <si>
+    <t>Emma Lewis</t>
+  </si>
+  <si>
+    <t>Mason Lee</t>
+  </si>
+  <si>
+    <t>Sophia Young</t>
+  </si>
+  <si>
+    <t>Alexander Walker</t>
+  </si>
+  <si>
+    <t>Harper Allen</t>
+  </si>
+  <si>
+    <t>Daniel King</t>
+  </si>
+  <si>
+    <t>Aria Wright</t>
+  </si>
+  <si>
+    <t>Henry Scott</t>
+  </si>
+  <si>
+    <t>Zoey Adams</t>
+  </si>
+  <si>
+    <t>Jackson Baker</t>
+  </si>
+  <si>
+    <t>Grace Nelson</t>
+  </si>
+  <si>
+    <t>Sebastian Hill</t>
+  </si>
+  <si>
+    <t>Natalie Turner</t>
+  </si>
+  <si>
+    <t>Aiden Phillips</t>
+  </si>
+  <si>
+    <t>Samantha Campbell</t>
+  </si>
+  <si>
+    <t>Gabriel Parker</t>
+  </si>
+  <si>
+    <t>Lily Evans</t>
+  </si>
+  <si>
+    <t>Christopher Edwards</t>
+  </si>
+  <si>
+    <t>Zoey Collins</t>
+  </si>
+  <si>
+    <t>Isaac Stewart</t>
+  </si>
+  <si>
+    <t>Chloe Sanchez</t>
+  </si>
+  <si>
+    <t>Nathan Morris</t>
+  </si>
+  <si>
+    <t>Madison Roberts</t>
+  </si>
+  <si>
+    <t>Lucas White</t>
+  </si>
+  <si>
+    <t>Ella Hall</t>
+  </si>
+  <si>
+    <t>fake_org_ceo_name</t>
+  </si>
+  <si>
+    <t>fake_contact_number</t>
+  </si>
+  <si>
+    <t>123-456-7890</t>
+  </si>
+  <si>
+    <t>987-654-3210</t>
+  </si>
+  <si>
+    <t>456-789-0123</t>
+  </si>
+  <si>
+    <t>789-012-3456</t>
+  </si>
+  <si>
+    <t>234-567-8901</t>
+  </si>
+  <si>
+    <t>678-901-2345</t>
+  </si>
+  <si>
+    <t>345-678-9012</t>
+  </si>
+  <si>
+    <t>890-123-4567</t>
+  </si>
+  <si>
+    <t>512-346-7890</t>
+  </si>
+  <si>
+    <t>403-257-8912</t>
+  </si>
+  <si>
+    <t>123-456-7891</t>
+  </si>
+  <si>
+    <t>987-654-3211</t>
+  </si>
+  <si>
+    <t>456-789-0124</t>
+  </si>
+  <si>
+    <t>789-012-3457</t>
+  </si>
+  <si>
+    <t>234-567-8902</t>
+  </si>
+  <si>
+    <t>678-901-2346</t>
+  </si>
+  <si>
+    <t>345-678-9013</t>
+  </si>
+  <si>
+    <t>890-123-4568</t>
+  </si>
+  <si>
+    <t>512-346-7891</t>
+  </si>
+  <si>
+    <t>403-257-8913</t>
+  </si>
+  <si>
+    <t>123-456-7892</t>
+  </si>
+  <si>
+    <t>987-654-3212</t>
+  </si>
+  <si>
+    <t>456-789-0125</t>
+  </si>
+  <si>
+    <t>789-012-3458</t>
+  </si>
+  <si>
+    <t>234-567-8903</t>
+  </si>
+  <si>
+    <t>678-901-2347</t>
+  </si>
+  <si>
+    <t>345-678-9014</t>
+  </si>
+  <si>
+    <t>890-123-4569</t>
+  </si>
+  <si>
+    <t>512-346-7892</t>
+  </si>
+  <si>
+    <t>403-257-8914</t>
+  </si>
+  <si>
+    <t>123-456-7893</t>
+  </si>
+  <si>
+    <t>987-654-3213</t>
+  </si>
+  <si>
+    <t>456-789-0126</t>
+  </si>
+  <si>
+    <t>789-012-3459</t>
+  </si>
+  <si>
+    <t>234-567-8904</t>
+  </si>
+  <si>
+    <t>678-901-2348</t>
+  </si>
+  <si>
+    <t>345-678-9015</t>
+  </si>
+  <si>
+    <t>890-123-4570</t>
+  </si>
+  <si>
+    <t>512-346-7893</t>
+  </si>
+  <si>
+    <t>403-257-8915</t>
+  </si>
+  <si>
+    <t>123-456-7894</t>
+  </si>
+  <si>
+    <t>987-654-3214</t>
+  </si>
+  <si>
+    <t>456-789-0127</t>
+  </si>
+  <si>
+    <t>789-012-3460</t>
+  </si>
+  <si>
+    <t>Finance</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -391,6 +664,26 @@
       <color rgb="FF1D1C1D"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1D1C1D"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -413,10 +706,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -731,16 +1027,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{788B024D-3CDE-B942-85CC-8359393F5746}">
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="55" customWidth="1"/>
     <col min="2" max="2" width="30.33203125" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" customWidth="1"/>
-    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="27.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>95</v>
       </c>
@@ -748,13 +1047,19 @@
         <v>73</v>
       </c>
       <c r="C1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="D1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -762,13 +1067,19 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" t="s">
         <v>72</v>
       </c>
-      <c r="D2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E2" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -776,13 +1087,19 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" t="s">
         <v>72</v>
       </c>
-      <c r="D3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E3" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -790,13 +1107,19 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" t="s">
         <v>72</v>
       </c>
-      <c r="D4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -804,13 +1127,19 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" t="s">
         <v>72</v>
       </c>
-      <c r="D5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E5" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -818,13 +1147,19 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" t="s">
         <v>72</v>
       </c>
-      <c r="D6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E6" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -832,13 +1167,19 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D7" t="s">
         <v>72</v>
       </c>
-      <c r="D7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E7" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
@@ -846,13 +1187,19 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8" t="s">
         <v>71</v>
       </c>
-      <c r="D8" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E8" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -860,13 +1207,19 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" t="s">
         <v>72</v>
       </c>
-      <c r="D9" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E9" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -874,13 +1227,19 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" t="s">
         <v>72</v>
       </c>
-      <c r="D10" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -888,13 +1247,19 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" t="s">
         <v>71</v>
       </c>
-      <c r="D11" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E11" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -902,13 +1267,19 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12" t="s">
         <v>72</v>
       </c>
-      <c r="D12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
@@ -916,13 +1287,19 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" t="s">
         <v>72</v>
       </c>
-      <c r="D13" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E13" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -930,13 +1307,19 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" t="s">
         <v>72</v>
       </c>
-      <c r="D14" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E14" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
@@ -944,13 +1327,19 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15" t="s">
         <v>72</v>
       </c>
-      <c r="D15" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E15" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
@@ -958,13 +1347,19 @@
         <v>29</v>
       </c>
       <c r="C16" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" t="s">
         <v>72</v>
       </c>
-      <c r="D16" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E16" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>30</v>
       </c>
@@ -972,13 +1367,19 @@
         <v>31</v>
       </c>
       <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="s">
         <v>72</v>
       </c>
-      <c r="D17" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E17" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -986,13 +1387,19 @@
         <v>33</v>
       </c>
       <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" t="s">
         <v>72</v>
       </c>
-      <c r="D18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E18" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
@@ -1000,13 +1407,19 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" t="s">
         <v>71</v>
       </c>
-      <c r="D19" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E19" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>96</v>
       </c>
@@ -1014,13 +1427,19 @@
         <v>36</v>
       </c>
       <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
         <v>72</v>
       </c>
-      <c r="D20" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E20" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>37</v>
       </c>
@@ -1028,13 +1447,19 @@
         <v>38</v>
       </c>
       <c r="C21" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" t="s">
         <v>72</v>
       </c>
-      <c r="D21" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E21" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>85</v>
       </c>
@@ -1042,13 +1467,19 @@
         <v>39</v>
       </c>
       <c r="C22" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" t="s">
         <v>69</v>
       </c>
-      <c r="D22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E22" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>86</v>
       </c>
@@ -1056,13 +1487,19 @@
         <v>40</v>
       </c>
       <c r="C23" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" t="s">
         <v>69</v>
       </c>
-      <c r="D23" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E23" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>41</v>
       </c>
@@ -1070,13 +1507,19 @@
         <v>42</v>
       </c>
       <c r="C24" t="s">
+        <v>103</v>
+      </c>
+      <c r="D24" t="s">
         <v>69</v>
       </c>
-      <c r="D24" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E24" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>87</v>
       </c>
@@ -1084,13 +1527,19 @@
         <v>43</v>
       </c>
       <c r="C25" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" t="s">
         <v>69</v>
       </c>
-      <c r="D25" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E25" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>88</v>
       </c>
@@ -1098,13 +1547,19 @@
         <v>44</v>
       </c>
       <c r="C26" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" t="s">
         <v>69</v>
       </c>
-      <c r="D26" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E26" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>89</v>
       </c>
@@ -1112,13 +1567,19 @@
         <v>40</v>
       </c>
       <c r="C27" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" t="s">
         <v>69</v>
       </c>
-      <c r="D27" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E27" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>90</v>
       </c>
@@ -1126,13 +1587,19 @@
         <v>91</v>
       </c>
       <c r="C28" t="s">
+        <v>100</v>
+      </c>
+      <c r="D28" t="s">
         <v>69</v>
       </c>
-      <c r="D28" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E28" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>45</v>
       </c>
@@ -1140,13 +1607,19 @@
         <v>46</v>
       </c>
       <c r="C29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" t="s">
         <v>69</v>
       </c>
-      <c r="D29" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E29" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>92</v>
       </c>
@@ -1154,13 +1627,19 @@
         <v>47</v>
       </c>
       <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" t="s">
         <v>69</v>
       </c>
-      <c r="D30" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E30" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>93</v>
       </c>
@@ -1168,13 +1647,19 @@
         <v>94</v>
       </c>
       <c r="C31" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" t="s">
         <v>69</v>
       </c>
-      <c r="D31" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E31" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>48</v>
       </c>
@@ -1182,13 +1667,19 @@
         <v>49</v>
       </c>
       <c r="C32" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32" t="s">
         <v>68</v>
       </c>
-      <c r="D32" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E32" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>50</v>
       </c>
@@ -1196,13 +1687,19 @@
         <v>51</v>
       </c>
       <c r="C33" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" t="s">
         <v>68</v>
       </c>
-      <c r="D33" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E33" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>52</v>
       </c>
@@ -1210,13 +1707,19 @@
         <v>53</v>
       </c>
       <c r="C34" t="s">
+        <v>101</v>
+      </c>
+      <c r="D34" t="s">
         <v>68</v>
       </c>
-      <c r="D34" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E34" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>54</v>
       </c>
@@ -1224,13 +1727,19 @@
         <v>55</v>
       </c>
       <c r="C35" t="s">
+        <v>100</v>
+      </c>
+      <c r="D35" t="s">
         <v>68</v>
       </c>
-      <c r="D35" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E35" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>56</v>
       </c>
@@ -1238,13 +1747,19 @@
         <v>57</v>
       </c>
       <c r="C36" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" t="s">
         <v>68</v>
       </c>
-      <c r="D36" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E36" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -1252,13 +1767,19 @@
         <v>59</v>
       </c>
       <c r="C37" t="s">
+        <v>100</v>
+      </c>
+      <c r="D37" t="s">
         <v>68</v>
       </c>
-      <c r="D37" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E37" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>60</v>
       </c>
@@ -1266,13 +1787,19 @@
         <v>61</v>
       </c>
       <c r="C38" t="s">
+        <v>98</v>
+      </c>
+      <c r="D38" t="s">
         <v>68</v>
       </c>
-      <c r="D38" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E38" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>62</v>
       </c>
@@ -1280,13 +1807,19 @@
         <v>63</v>
       </c>
       <c r="C39" t="s">
+        <v>102</v>
+      </c>
+      <c r="D39" t="s">
         <v>68</v>
       </c>
-      <c r="D39" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E39" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>64</v>
       </c>
@@ -1294,13 +1827,19 @@
         <v>65</v>
       </c>
       <c r="C40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D40" t="s">
         <v>68</v>
       </c>
-      <c r="D40" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E40" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>66</v>
       </c>
@@ -1308,13 +1847,19 @@
         <v>67</v>
       </c>
       <c r="C41" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" t="s">
         <v>68</v>
       </c>
-      <c r="D41" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="E41" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>74</v>
       </c>
@@ -1322,13 +1867,19 @@
         <v>75</v>
       </c>
       <c r="C42" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="D42" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+        <v>202</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>76</v>
       </c>
@@ -1336,13 +1887,19 @@
         <v>77</v>
       </c>
       <c r="C43" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="D43" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+        <v>202</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>78</v>
       </c>
@@ -1350,13 +1907,19 @@
         <v>79</v>
       </c>
       <c r="C44" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="D44" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+        <v>202</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>80</v>
       </c>
@@ -1364,13 +1927,20 @@
         <v>81</v>
       </c>
       <c r="C45" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="D45" t="s">
-        <v>101</v>
+        <v>202</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
lots of formatting changes, added in section for data quality and methods etc. tried adding in logo but proving fiddly for time being - to go back and fix next week
</commit_message>
<xml_diff>
--- a/orgs_test/2023-11-21 fictional_orgs_list.xlsx
+++ b/orgs_test/2023-11-21 fictional_orgs_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin.ingram/Martin Ingram R Work/martin-ingram.github.io/orgs_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD0818C-9DA2-2F47-BED3-3B0438EE9D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA87AADC-0B9B-6444-9CD1-41CCCF7C8FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" xr2:uid="{9B7B9A65-6A20-384F-90D3-B47F15698559}"/>
+    <workbookView xWindow="-40260" yWindow="2160" windowWidth="30240" windowHeight="17200" xr2:uid="{9B7B9A65-6A20-384F-90D3-B47F15698559}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="201">
   <si>
     <t>Stark Industries</t>
   </si>
@@ -167,15 +167,9 @@
     <t>TV Show - Suits</t>
   </si>
   <si>
-    <t>TV Show - Boston Legal</t>
-  </si>
-  <si>
     <t>Comic/TV Show - Daredevil</t>
   </si>
   <si>
-    <t>Goliath National Bank Legal</t>
-  </si>
-  <si>
     <t>TV Show - How I Met Your Mother</t>
   </si>
   <si>
@@ -242,21 +236,9 @@
     <t>TV Show - Chicago Hope</t>
   </si>
   <si>
-    <t>Medical</t>
-  </si>
-  <si>
-    <t>Legal</t>
-  </si>
-  <si>
     <t>classification</t>
   </si>
   <si>
-    <t>Commercial</t>
-  </si>
-  <si>
-    <t>Research and Development</t>
-  </si>
-  <si>
     <t>source</t>
   </si>
   <si>
@@ -644,7 +626,19 @@
     <t>789-012-3460</t>
   </si>
   <si>
-    <t>Finance</t>
+    <t>Agency</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>External Body</t>
+  </si>
+  <si>
+    <t>TV Show - Boston External Body</t>
+  </si>
+  <si>
+    <t>Goliath National Bank External Body</t>
   </si>
 </sst>
 </file>
@@ -706,12 +700,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1041,22 +1034,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="F1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1067,16 +1060,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>158</v>
+        <v>106</v>
+      </c>
+      <c r="F2" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1087,16 +1080,16 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>159</v>
+        <v>107</v>
+      </c>
+      <c r="F3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1107,16 +1100,16 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>160</v>
+        <v>108</v>
+      </c>
+      <c r="F4" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1127,16 +1120,16 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>161</v>
+        <v>109</v>
+      </c>
+      <c r="F5" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1147,16 +1140,16 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>162</v>
+        <v>110</v>
+      </c>
+      <c r="F6" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1167,16 +1160,16 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>163</v>
+        <v>111</v>
+      </c>
+      <c r="F7" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1187,16 +1180,16 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D8" t="s">
-        <v>71</v>
+        <v>198</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>164</v>
+        <v>112</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1207,16 +1200,16 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>165</v>
+        <v>113</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1227,16 +1220,16 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>166</v>
+        <v>114</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1247,16 +1240,16 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>198</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>167</v>
+        <v>115</v>
+      </c>
+      <c r="F11" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1267,16 +1260,16 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D12" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>168</v>
+        <v>116</v>
+      </c>
+      <c r="F12" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1287,16 +1280,16 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>169</v>
+        <v>117</v>
+      </c>
+      <c r="F13" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1307,16 +1300,16 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>170</v>
+        <v>118</v>
+      </c>
+      <c r="F14" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1327,16 +1320,16 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D15" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>171</v>
+        <v>119</v>
+      </c>
+      <c r="F15" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1347,16 +1340,16 @@
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>172</v>
+        <v>120</v>
+      </c>
+      <c r="F16" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1367,16 +1360,16 @@
         <v>31</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>173</v>
+        <v>121</v>
+      </c>
+      <c r="F17" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1387,16 +1380,16 @@
         <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>174</v>
+        <v>122</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1407,36 +1400,36 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>198</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>175</v>
+        <v>123</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B20" t="s">
         <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>176</v>
+        <v>124</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1447,56 +1440,56 @@
         <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>177</v>
+        <v>125</v>
+      </c>
+      <c r="F21" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
         <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D22" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>178</v>
+        <v>126</v>
+      </c>
+      <c r="F22" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
         <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D23" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>179</v>
+        <v>127</v>
+      </c>
+      <c r="F23" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="20" x14ac:dyDescent="0.25">
@@ -1507,436 +1500,436 @@
         <v>42</v>
       </c>
       <c r="C24" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>180</v>
+        <v>128</v>
+      </c>
+      <c r="F24" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>199</v>
       </c>
       <c r="C25" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D25" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>181</v>
+        <v>129</v>
+      </c>
+      <c r="F25" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C26" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D26" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>182</v>
+        <v>130</v>
+      </c>
+      <c r="F26" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B27" t="s">
         <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D27" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>183</v>
+        <v>131</v>
+      </c>
+      <c r="F27" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>184</v>
+        <v>132</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>45</v>
+        <v>200</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>185</v>
+        <v>133</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B30" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C30" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D30" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>186</v>
+        <v>134</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B31" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C31" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D31" t="s">
-        <v>69</v>
+        <v>198</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>187</v>
+        <v>135</v>
+      </c>
+      <c r="F31" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D32" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>188</v>
+        <v>136</v>
+      </c>
+      <c r="F32" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C33" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D33" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>189</v>
+        <v>137</v>
+      </c>
+      <c r="F33" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B34" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C34" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
+      </c>
+      <c r="F34" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D35" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>191</v>
+        <v>139</v>
+      </c>
+      <c r="F35" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C36" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>192</v>
+        <v>140</v>
+      </c>
+      <c r="F36" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B37" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C37" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D37" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>193</v>
+        <v>141</v>
+      </c>
+      <c r="F37" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B38" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C38" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D38" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>194</v>
+        <v>142</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B39" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C39" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D39" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>195</v>
+        <v>143</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B40" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C40" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D40" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>196</v>
+        <v>144</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B41" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C41" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D41" t="s">
-        <v>68</v>
+        <v>197</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>197</v>
+        <v>145</v>
+      </c>
+      <c r="F41" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C42" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>198</v>
+        <v>146</v>
+      </c>
+      <c r="F42" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D43" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>199</v>
+        <v>147</v>
+      </c>
+      <c r="F43" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B44" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C44" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D44" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>200</v>
+        <v>148</v>
+      </c>
+      <c r="F44" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D45" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>201</v>
+        <v>149</v>
+      </c>
+      <c r="F45" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -1955,57 +1948,57 @@
   <sheetData>
     <row r="1" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" t="s">
         <v>78</v>
-      </c>
-      <c r="B3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
fixed incorrect org names
</commit_message>
<xml_diff>
--- a/orgs_test/2023-11-21 fictional_orgs_list.xlsx
+++ b/orgs_test/2023-11-21 fictional_orgs_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin.ingram/Martin Ingram R Work/martin-ingram.github.io/orgs_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA87AADC-0B9B-6444-9CD1-41CCCF7C8FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C55893-9506-5B4C-ABEC-3D5CF76F1751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-40260" yWindow="2160" windowWidth="30240" windowHeight="17200" xr2:uid="{9B7B9A65-6A20-384F-90D3-B47F15698559}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17180" xr2:uid="{9B7B9A65-6A20-384F-90D3-B47F15698559}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -635,10 +635,10 @@
     <t>External Body</t>
   </si>
   <si>
-    <t>TV Show - Boston External Body</t>
-  </si>
-  <si>
-    <t>Goliath National Bank External Body</t>
+    <t>Goliath National Bank Legal</t>
+  </si>
+  <si>
+    <t>TV Show - Boston Legal</t>
   </si>
 </sst>
 </file>
@@ -1517,7 +1517,7 @@
         <v>81</v>
       </c>
       <c r="B25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C25" t="s">
         <v>92</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="29" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B29" t="s">
         <v>44</v>

</xml_diff>